<commit_message>
added: some questions + cp31
</commit_message>
<xml_diff>
--- a/SPEP/CompetiQuest.xlsx
+++ b/SPEP/CompetiQuest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\cph\SPEP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DF03A2-98F7-4A8C-899B-B4641A9BA6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D4D1823-37EF-4199-9102-3302943016BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11295" xr2:uid="{BDEB6F72-BEEF-4BC5-8CFA-D895C7732EBD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BDEB6F72-BEEF-4BC5-8CFA-D895C7732EBD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="261">
   <si>
     <t>Serial No.</t>
   </si>
@@ -795,6 +798,30 @@
   </si>
   <si>
     <t>https://www.interviewbit.com/problems/shortest-unique-prefix/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/robot-bounded-in-circle/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/average-waiting-time/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-distance-to-the-target-element/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-size-subarray-in-infinite-array/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/split-a-string-in-balanced-strings/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/cherry-pickup/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/avoid-flood-in-the-city/description/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/most-stones-removed-with-same-row-or-column/description/</t>
   </si>
 </sst>
 </file>
@@ -1288,9 +1315,6 @@
       <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
@@ -1380,6 +1404,9 @@
       </c>
       <c r="B18" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -3307,47 +3334,71 @@
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
+      <c r="B217" s="3" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="1">
         <f t="shared" si="3"/>
         <v>217</v>
       </c>
+      <c r="B218" s="3" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="1">
         <f t="shared" si="3"/>
         <v>218</v>
       </c>
+      <c r="B219" s="3" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="1">
         <f t="shared" si="3"/>
         <v>219</v>
       </c>
+      <c r="B220" s="3" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="1">
         <f t="shared" si="3"/>
         <v>220</v>
       </c>
+      <c r="B221" s="3" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="1">
         <f t="shared" si="3"/>
         <v>221</v>
       </c>
+      <c r="B222" s="3" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <f t="shared" si="3"/>
         <v>222</v>
       </c>
+      <c r="B223" s="3" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="1">
         <f t="shared" si="3"/>
         <v>223</v>
+      </c>
+      <c r="B224" s="3" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.25">
@@ -4047,6 +4098,14 @@
     <hyperlink ref="B212" r:id="rId231" xr:uid="{BA19BE7D-72F6-41CE-96B7-EDB37331BDA0}"/>
     <hyperlink ref="B213" r:id="rId232" xr:uid="{2DEE5BFA-952D-4FAF-A1A9-5DD0CF46EAA2}"/>
     <hyperlink ref="B214" r:id="rId233" xr:uid="{C2B073D2-0C8A-4F10-98F6-CFC8891493B2}"/>
+    <hyperlink ref="B217" r:id="rId234" xr:uid="{61DB6CEC-1CDD-4311-A132-772A5CFDE7A0}"/>
+    <hyperlink ref="B218" r:id="rId235" xr:uid="{9452EB98-B937-4E64-AF2D-9ADA05AE1445}"/>
+    <hyperlink ref="B219" r:id="rId236" xr:uid="{89E9654A-7ABE-497A-9780-E93F60430A72}"/>
+    <hyperlink ref="B220" r:id="rId237" xr:uid="{9D51E878-E496-4D4E-98FA-0AAAA0F6CE48}"/>
+    <hyperlink ref="B221" r:id="rId238" xr:uid="{AFB14665-DD42-405E-9AA6-A9691370F8B5}"/>
+    <hyperlink ref="B222" r:id="rId239" xr:uid="{508FD289-CA41-42CC-B7DD-097173BDFCB6}"/>
+    <hyperlink ref="B223" r:id="rId240" xr:uid="{603760A7-D3A3-4332-A254-5FD589E94FE9}"/>
+    <hyperlink ref="B224" r:id="rId241" xr:uid="{EF3F751D-B048-465F-A729-59910E0634E6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>